<commit_message>
docs: regenerate logic spec Excel v1.5
</commit_message>
<xml_diff>
--- a/Specs/LOGIC_SPEC-v1.xlsx
+++ b/Specs/LOGIC_SPEC-v1.xlsx
@@ -844,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -902,107 +902,115 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>3. Overpayments *(resolved in v175+)*</t>
+          <t>3. Overpayments *(resolved in v175+; simplified in v290)*</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>- `Crud.save()` / `bulkSave()` now reject `paid_amount &gt; amount` for transactions and procurements server-side.</t>
+          <t>- `Crud.save()` / `bulkSave()` reject `paid_amount &gt; amount` server-side.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>- Project expense no longer exposes `paid_amount` to the user; it is always set equal to `amount`. Vendor payments are handled separately via `vendor_settlement`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>4. Credit vs. immediate vs. settlement</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>- Payment term is inferred from amount/paid comparison. It is not independently validated against the paid amount.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>5. Employee module (on hold)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>- Payroll, attendance, and custody RLS policies are currently open because the module is disabled.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
+          <t>- Payroll, attendance, and custody RLS policies are currently open because the module is disabled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
           <t>- When enabled, these must follow the same owner/admin permission model.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>6. Retention / holdback (ضمان الأعمال)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>- Not implemented. Decide whether retention should be a separate transaction type, a project-level field, or an invoice line-item deduction.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>7. Password-reset email delivery verification</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>- The new `admin_reset_password_email` RPC (v289) enqueues the email via `pg_net`. The RPC returns success immediately; actual Resend delivery status must be checked in Resend logs or `net._http_response`.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
+          <t>- The new `admin_reset_password_email` RPC (v289) enqueues the email via `pg_net`. The RPC returns success immediately; actual Resend delivery status must be checked in Resend logs or `net._http_response`.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="19">
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A11:H11"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A16:H16"/>
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="A18:H18"/>
-    <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A3:H3"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A11:H11"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A6:H6"/>
     <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A19:H19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1256,7 +1264,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Version: 1.3</t>
+          <t>Version: 1.5</t>
         </is>
       </c>
     </row>
@@ -1270,7 +1278,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Updated: 2026-07-06</t>
+          <t>Updated: 2026-07-08</t>
         </is>
       </c>
     </row>
@@ -1624,198 +1632,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="80" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ch2 Project Accounting</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>2.1 Project Inputs</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>For a single project, gather all its live (non-deleted) transactions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>Project Deposits  = Σ Amount of all project_deposit transactions
-Project Expenses  = Σ Amount of all project_expense transactions
-Design Expenses   = Σ Amount of project_expense where category = design
-Construction Exp. = Project Expenses − Design Expenses</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>2.2 Supervision Fee</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Supervision is a fee the office earns as a percentage of construction-related expenses only. Design costs are excluded from the base.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Supervision Fee = Construction Expenses × (Supervision % / 100)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Where `Supervision %` is set on the project master record.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Important: Supervision is computed on demand and is not stored as a separate transaction row. It affects project net balance and office income, but it does not appear directly in the transaction list unless a manual supervision transaction is created.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>2.3 Project Net Balance</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Project Net Balance = Project Deposits − Project Expenses − Supervision Fee</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Interpretation:</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Positive → client still owes money (deposits exceed costs + fee).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Zero → account is square.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Negative → project is over-budget or over-paid by the client.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>2.4 Client Balance</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>A client may have many projects. The client balance is the sum of the net balances of all client projects, with supervision applied consistently everywhere:</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>Client Deposits    = Σ Project Deposits     (for all client projects)
-Client Expenses    = Σ Project Expenses     (for all client projects)
-Client Supervision = Σ Supervision Fee      (for all client projects)
-Client Balance     = Client Deposits − Client Expenses − Client Supervision</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>The same supervision formula is applied consistently in project detail, client detail, client list, and dashboard active-client balances. The canonical view `client_balances` enforces this formula.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="20">
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A11:H11"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A18:H18"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A17:H17"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A19:H19"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1832,144 +1648,146 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ch3 Vendor Accounting</t>
+          <t>Ch2 Project Accounting</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>A vendor can supply two things:</t>
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>2.1 Project Inputs</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>1. Services → recorded directly as `project_expense` with the vendor linked.</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>For a single project, gather all its live (non-deleted) transactions:</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>2. Merchandise / Materials → recorded first as a `procurement`, which auto-creates a linked `project_expense` transaction.</t>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Project Deposits  = Σ Amount of all project_deposit transactions
+Project Expenses  = Σ Amount of all project_expense transactions
+Design Expenses   = Σ Amount of project_expense where category = design
+Construction Exp. = Project Expenses − Design Expenses</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>3.1 Vendor Owed</t>
+          <t>2.2 Supervision Fee</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Service Owed    = Σ Amount of project_expense rows linked to the vendor
-Merchandise Owed= Σ Total Price of procurement rows linked to the vendor
-Total Owed      = Service Owed + Merchandise Owed</t>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Supervision is a fee the office earns as a percentage of construction-related expenses only. Design costs are excluded from the base.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>3.2 Vendor Paid</t>
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Supervision Fee = Construction Expenses × (Supervision % / 100)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Service Paid    = Σ Paid Amount of those service project_expense rows
-Merchandise Paid= Σ Paid Amount of those procurements
-Total Paid      = Service Paid + Merchandise Paid</t>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Where `Supervision %` is set on the project master record.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>3.3 Vendor Balance</t>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Important: Supervision is computed on demand and is not stored as a separate transaction row. It affects project net balance and office income, but it does not appear directly in the transaction list unless a manual supervision transaction is created.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Vendor Balance = Total Owed − Total Paid</t>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>2.3 Project Net Balance</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Project Net Balance = Project Deposits − Project Expenses − Supervision Fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Interpretation:</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Positive → office still owes the vendor.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Zero → fully paid.</t>
+          <t>Positive → client still owes money (deposits exceed costs + fee).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Negative → vendor was over-paid.</t>
+          <t>Zero → account is square.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>3.4 Office Vendor</t>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Negative → project is over-budget or over-paid by the client.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>The system seeds one special vendor marked `is_office = true` (e.g. "مكتب سارة أبو العلا"). This vendor represents the office itself and can be used for:</t>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Project expenses are treated as fully paid. The `paid_amount` field is not collected on the project expense form; `paid_amount` is set equal to `amount` and `payment_term` is set to `immediate`. Any subsequent payment to the vendor is recorded separately as a project-agnostic `vendor_settlement` from the vendors screen.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Project expenses where the office is the service provider.</t>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>2.4 Client Balance</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Procurements where the office is the supplier.</t>
+          <t>A client may have many projects. The client balance is the sum of the net balances of all client projects, with supervision applied consistently everywhere:</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Office expenses linked to a vendor for traceability.</t>
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Client Deposits    = Σ Project Deposits     (for all client projects)
+Client Expenses    = Σ Project Expenses     (for all client projects)
+Client Supervision = Σ Supervision Fee      (for all client projects)
+Client Balance     = Client Deposits − Client Expenses − Client Supervision</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Transactions linked to the office vendor are included in vendor balances and the top-vendor dashboard like any other vendor. Their paid amounts are also still treated as office income and appear in the office cash-flow.</t>
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>The same supervision formula is applied consistently in project detail, client detail, client list, and dashboard active-client balances. The canonical view `client_balances` enforces this formula.</t>
         </is>
       </c>
     </row>
@@ -2008,6 +1826,276 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="80" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ch3 Vendor Accounting</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>A vendor can supply two things:</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>1. Services → recorded directly as `project_expense` with the vendor linked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>2. Merchandise / Materials → recorded first as a `procurement`, which auto-creates a linked `project_expense` transaction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Since v290, cost recognition and cash settlement are separated:</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>`project_expense` rows record that a cost was incurred (accrual).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>`vendor_settlement` rows record actual cash paid to the vendor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>`procurement` rows still track their own `paid_amount` because they function as purchase orders with their own payment lifecycle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>3.1 Vendor Owed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Service Owed     = Σ Amount of project_expense rows linked to the vendor
+Merchandise Owed = Σ Total Price of procurement rows linked to the vendor
+Total Owed       = Service Owed + Merchandise Owed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>3.2 Vendor Paid</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Service Paid     = Σ Paid Amount of vendor_settlement rows linked to the vendor
+Merchandise Paid = Σ Paid Amount of procurement rows linked to the vendor
+Total Paid       = Service Paid + Merchandise Paid</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>3.3 Vendor Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Vendor Balance = Total Owed − Total Paid</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Interpretation:</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Positive → office still owes the vendor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Zero → fully paid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Negative → vendor was over-paid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>3.4 vendor_settlement Rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Linked to a vendor only; no project is required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Represent cash leaving the office to the vendor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Can be entered from the vendors screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Reduce the vendor balance immediately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>3.5 Office Vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>The system seeds one special vendor marked `is_office = true` (e.g. "مكتب سارة أبو العلا"). This vendor represents the office itself and can be used for:</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Project expenses where the office is the service provider.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Procurements where the office is the supplier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Office expenses linked to a vendor for traceability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Transactions linked to the office vendor are included in vendor balances and the top-vendor dashboard like any other vendor. Their paid amounts are also still treated as office income and appear in the office cash-flow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="30">
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A19:H19"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2148,7 +2236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -2215,42 +2303,49 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>This linked row is used for project cash-flow and balance calculations. The vendor's overall balance, however, is computed from the procurement's own `paid_amount` plus any `vendor_settlement` rows linked to the vendor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>5.3 Consistency Rules</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Editing the procurement updates the linked transaction.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Deleting the procurement soft-deletes the linked transaction.</t>
+          <t>Editing the procurement updates the linked transaction.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>A procurement with no project has no linked transaction (it does not affect project balance).</t>
+          <t>Deleting the procurement soft-deletes the linked transaction.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
+          <t>A procurement with no project has no linked transaction (it does not affect project balance).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A9:H9"/>
@@ -2259,6 +2354,7 @@
     <mergeCell ref="A7:H7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A13:H13"/>
     <mergeCell ref="A11:H11"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A8:H8"/>

</xml_diff>